<commit_message>
feat: split melatonin into MT1, MT2 and Melatonin (3 products)
Price sheet now lists MT2 (\$60), MT1 (\$60) and Melatonin
(\$80) as three separate SKUs. Adding MT2 and MT1 as standalone
products with their own images from 素材/产品图片/Melatonin/.

Melatonin's price corrected from \$60 to \$80 to match the
high-dose MT10 entry in the sheet.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/素材/价格表.xlsx
+++ b/素材/价格表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11480"/>
+    <workbookView windowHeight="15080"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="233">
   <si>
     <t>Product name</t>
   </si>
@@ -506,13 +506,13 @@
     <t>MS40</t>
   </si>
   <si>
+    <t>MT2</t>
+  </si>
+  <si>
+    <t>MT1</t>
+  </si>
+  <si>
     <t>Melatonin</t>
-  </si>
-  <si>
-    <t>MT2</t>
-  </si>
-  <si>
-    <t>MT1</t>
   </si>
   <si>
     <t>MT10</t>
@@ -1776,7 +1776,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1951,12 +1951,6 @@
     <xf numFmtId="0" fontId="2" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1970,9 +1964,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3932,11 +3923,13 @@
         <v>60</v>
       </c>
       <c r="D93" s="10" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1" spans="1:4">
+      <c r="A94" s="55" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="94" ht="20" customHeight="1" spans="1:4">
-      <c r="A94" s="58"/>
       <c r="B94" s="56" t="s">
         <v>8</v>
       </c>
@@ -3944,11 +3937,13 @@
         <v>60</v>
       </c>
       <c r="D94" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="95" customHeight="1" spans="1:4">
+      <c r="A95" s="55" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="95" customHeight="1" spans="1:4">
-      <c r="A95" s="59"/>
       <c r="B95" s="56" t="s">
         <v>8</v>
       </c>
@@ -3960,13 +3955,13 @@
       </c>
     </row>
     <row r="96" customHeight="1" spans="1:4">
-      <c r="A96" s="60" t="s">
+      <c r="A96" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="B96" s="61" t="s">
+      <c r="B96" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="C96" s="62">
+      <c r="C96" s="60">
         <v>100</v>
       </c>
       <c r="D96" s="10" t="s">
@@ -3974,11 +3969,11 @@
       </c>
     </row>
     <row r="97" customHeight="1" spans="1:4">
-      <c r="A97" s="63"/>
-      <c r="B97" s="61" t="s">
+      <c r="A97" s="61"/>
+      <c r="B97" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C97" s="62">
+      <c r="C97" s="60">
         <v>170</v>
       </c>
       <c r="D97" s="10" t="s">
@@ -3986,13 +3981,13 @@
       </c>
     </row>
     <row r="98" customHeight="1" spans="1:4">
-      <c r="A98" s="64" t="s">
+      <c r="A98" s="62" t="s">
         <v>159</v>
       </c>
-      <c r="B98" s="61" t="s">
+      <c r="B98" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="C98" s="62">
+      <c r="C98" s="60">
         <v>45</v>
       </c>
       <c r="D98" s="32" t="s">
@@ -4000,11 +3995,11 @@
       </c>
     </row>
     <row r="99" customHeight="1" spans="1:4">
-      <c r="A99" s="63"/>
-      <c r="B99" s="61" t="s">
+      <c r="A99" s="61"/>
+      <c r="B99" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C99" s="62">
+      <c r="C99" s="60">
         <v>65</v>
       </c>
       <c r="D99" s="32" t="s">
@@ -4012,13 +4007,13 @@
       </c>
     </row>
     <row r="100" ht="20" customHeight="1" spans="1:4">
-      <c r="A100" s="61" t="s">
+      <c r="A100" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="B100" s="61" t="s">
+      <c r="B100" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C100" s="62">
+      <c r="C100" s="60">
         <v>65</v>
       </c>
       <c r="D100" s="10" t="s">
@@ -4026,13 +4021,13 @@
       </c>
     </row>
     <row r="101" customHeight="1" spans="1:4">
-      <c r="A101" s="64" t="s">
+      <c r="A101" s="62" t="s">
         <v>164</v>
       </c>
-      <c r="B101" s="61" t="s">
+      <c r="B101" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="C101" s="62">
+      <c r="C101" s="60">
         <v>45</v>
       </c>
       <c r="D101" s="10" t="s">
@@ -4040,11 +4035,11 @@
       </c>
     </row>
     <row r="102" customHeight="1" spans="1:4">
-      <c r="A102" s="63"/>
-      <c r="B102" s="61" t="s">
+      <c r="A102" s="61"/>
+      <c r="B102" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C102" s="62">
+      <c r="C102" s="60">
         <v>65</v>
       </c>
       <c r="D102" s="10" t="s">
@@ -4052,13 +4047,13 @@
       </c>
     </row>
     <row r="103" customHeight="1" spans="1:4">
-      <c r="A103" s="64" t="s">
+      <c r="A103" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="B103" s="61" t="s">
+      <c r="B103" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="C103" s="62">
+      <c r="C103" s="60">
         <v>50</v>
       </c>
       <c r="D103" s="10" t="s">
@@ -4066,11 +4061,11 @@
       </c>
     </row>
     <row r="104" customHeight="1" spans="1:4">
-      <c r="A104" s="63"/>
-      <c r="B104" s="61" t="s">
+      <c r="A104" s="61"/>
+      <c r="B104" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C104" s="62">
+      <c r="C104" s="60">
         <v>65</v>
       </c>
       <c r="D104" s="10" t="s">
@@ -4078,13 +4073,13 @@
       </c>
     </row>
     <row r="105" customHeight="1" spans="1:4">
-      <c r="A105" s="64" t="s">
+      <c r="A105" s="62" t="s">
         <v>170</v>
       </c>
-      <c r="B105" s="61" t="s">
+      <c r="B105" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C105" s="62">
+      <c r="C105" s="60">
         <v>90</v>
       </c>
       <c r="D105" s="10" t="s">
@@ -4092,11 +4087,11 @@
       </c>
     </row>
     <row r="106" customHeight="1" spans="1:4">
-      <c r="A106" s="60"/>
-      <c r="B106" s="61" t="s">
+      <c r="A106" s="58"/>
+      <c r="B106" s="59" t="s">
         <v>172</v>
       </c>
-      <c r="C106" s="62">
+      <c r="C106" s="60">
         <v>223</v>
       </c>
       <c r="D106" s="10" t="s">
@@ -4104,11 +4099,11 @@
       </c>
     </row>
     <row r="107" customHeight="1" spans="1:4">
-      <c r="A107" s="63"/>
-      <c r="B107" s="61" t="s">
+      <c r="A107" s="61"/>
+      <c r="B107" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="C107" s="62">
+      <c r="C107" s="60">
         <v>340</v>
       </c>
       <c r="D107" s="10" t="s">
@@ -4116,13 +4111,13 @@
       </c>
     </row>
     <row r="108" customHeight="1" spans="1:4">
-      <c r="A108" s="61" t="s">
+      <c r="A108" s="59" t="s">
         <v>175</v>
       </c>
-      <c r="B108" s="61" t="s">
+      <c r="B108" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="C108" s="62">
+      <c r="C108" s="60">
         <v>100</v>
       </c>
       <c r="D108" s="10">
@@ -4130,11 +4125,11 @@
       </c>
     </row>
     <row r="109" customHeight="1" spans="1:4">
-      <c r="A109" s="61"/>
-      <c r="B109" s="61" t="s">
+      <c r="A109" s="59"/>
+      <c r="B109" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="C109" s="62">
+      <c r="C109" s="60">
         <v>153</v>
       </c>
       <c r="D109" s="10">
@@ -4156,7 +4151,7 @@
       </c>
     </row>
     <row r="111" ht="22" customHeight="1" spans="1:4">
-      <c r="A111" s="65" t="s">
+      <c r="A111" s="55" t="s">
         <v>178</v>
       </c>
       <c r="B111" s="56" t="s">
@@ -4168,7 +4163,7 @@
       <c r="D111" s="10"/>
     </row>
     <row r="112" customHeight="1" spans="1:5">
-      <c r="A112" s="65" t="s">
+      <c r="A112" s="55" t="s">
         <v>180</v>
       </c>
       <c r="B112" s="56" t="s">
@@ -4185,7 +4180,7 @@
       </c>
     </row>
     <row r="113" customHeight="1" spans="1:4">
-      <c r="A113" s="66"/>
+      <c r="A113" s="63"/>
       <c r="B113" s="56" t="s">
         <v>8</v>
       </c>
@@ -4197,7 +4192,7 @@
       </c>
     </row>
     <row r="114" customHeight="1" spans="1:4">
-      <c r="A114" s="65" t="s">
+      <c r="A114" s="55" t="s">
         <v>184</v>
       </c>
       <c r="B114" s="56" t="s">
@@ -4211,7 +4206,7 @@
       </c>
     </row>
     <row r="115" customHeight="1" spans="1:4">
-      <c r="A115" s="66"/>
+      <c r="A115" s="63"/>
       <c r="B115" s="56" t="s">
         <v>8</v>
       </c>
@@ -4223,7 +4218,7 @@
       </c>
     </row>
     <row r="116" customHeight="1" spans="1:4">
-      <c r="A116" s="67" t="s">
+      <c r="A116" s="64" t="s">
         <v>187</v>
       </c>
       <c r="B116" s="56" t="s">
@@ -4237,7 +4232,7 @@
       </c>
     </row>
     <row r="117" customHeight="1" spans="1:4">
-      <c r="A117" s="68"/>
+      <c r="A117" s="65"/>
       <c r="B117" s="56" t="s">
         <v>8</v>
       </c>
@@ -4249,7 +4244,7 @@
       </c>
     </row>
     <row r="118" customHeight="1" spans="1:4">
-      <c r="A118" s="68"/>
+      <c r="A118" s="65"/>
       <c r="B118" s="56" t="s">
         <v>18</v>
       </c>
@@ -4275,7 +4270,7 @@
       </c>
     </row>
     <row r="120" ht="22" customHeight="1" spans="1:4">
-      <c r="A120" s="65" t="s">
+      <c r="A120" s="55" t="s">
         <v>193</v>
       </c>
       <c r="B120" s="56" t="s">
@@ -4287,7 +4282,7 @@
       <c r="D120" s="10"/>
     </row>
     <row r="121" customHeight="1" spans="1:4">
-      <c r="A121" s="65" t="s">
+      <c r="A121" s="55" t="s">
         <v>194</v>
       </c>
       <c r="B121" s="56" t="s">
@@ -4301,7 +4296,7 @@
       </c>
     </row>
     <row r="122" customHeight="1" spans="1:4">
-      <c r="A122" s="66"/>
+      <c r="A122" s="63"/>
       <c r="B122" s="56" t="s">
         <v>8</v>
       </c>
@@ -4313,7 +4308,7 @@
       </c>
     </row>
     <row r="123" customHeight="1" spans="1:4">
-      <c r="A123" s="65" t="s">
+      <c r="A123" s="55" t="s">
         <v>197</v>
       </c>
       <c r="B123" s="56" t="s">
@@ -4327,7 +4322,7 @@
       </c>
     </row>
     <row r="124" customHeight="1" spans="1:4">
-      <c r="A124" s="66"/>
+      <c r="A124" s="63"/>
       <c r="B124" s="56" t="s">
         <v>8</v>
       </c>
@@ -4339,7 +4334,7 @@
       </c>
     </row>
     <row r="125" customHeight="1" spans="1:4">
-      <c r="A125" s="69" t="s">
+      <c r="A125" s="66" t="s">
         <v>200</v>
       </c>
       <c r="B125" s="56" t="s">
@@ -4353,7 +4348,7 @@
       </c>
     </row>
     <row r="126" customHeight="1" spans="1:4">
-      <c r="A126" s="70"/>
+      <c r="A126" s="67"/>
       <c r="B126" s="56" t="s">
         <v>8</v>
       </c>
@@ -4365,19 +4360,19 @@
       </c>
     </row>
     <row r="127" customHeight="1" spans="1:4">
-      <c r="A127" s="71"/>
-      <c r="B127" s="72"/>
-      <c r="C127" s="72"/>
-      <c r="D127" s="73"/>
+      <c r="A127" s="68"/>
+      <c r="B127" s="69"/>
+      <c r="C127" s="69"/>
+      <c r="D127" s="70"/>
     </row>
     <row r="128" customHeight="1" spans="1:4">
-      <c r="A128" s="74" t="s">
+      <c r="A128" s="71" t="s">
         <v>203</v>
       </c>
-      <c r="B128" s="74" t="s">
+      <c r="B128" s="71" t="s">
         <v>204</v>
       </c>
-      <c r="C128" s="75">
+      <c r="C128" s="72">
         <v>185</v>
       </c>
       <c r="D128" s="10" t="s">
@@ -4385,13 +4380,13 @@
       </c>
     </row>
     <row r="129" customHeight="1" spans="1:4">
-      <c r="A129" s="76" t="s">
+      <c r="A129" s="73" t="s">
         <v>206</v>
       </c>
-      <c r="B129" s="77" t="s">
+      <c r="B129" s="74" t="s">
         <v>204</v>
       </c>
-      <c r="C129" s="78">
+      <c r="C129" s="75">
         <v>120</v>
       </c>
       <c r="D129" s="10" t="s">
@@ -4399,11 +4394,11 @@
       </c>
     </row>
     <row r="130" customHeight="1" spans="1:4">
-      <c r="A130" s="74"/>
-      <c r="B130" s="77" t="s">
+      <c r="A130" s="71"/>
+      <c r="B130" s="74" t="s">
         <v>208</v>
       </c>
-      <c r="C130" s="78">
+      <c r="C130" s="75">
         <v>195</v>
       </c>
       <c r="D130" s="10" t="s">
@@ -4411,19 +4406,19 @@
       </c>
     </row>
     <row r="131" hidden="1" customHeight="1" spans="1:4">
-      <c r="A131" s="79"/>
-      <c r="B131" s="79"/>
-      <c r="C131" s="75"/>
+      <c r="A131" s="76"/>
+      <c r="B131" s="76"/>
+      <c r="C131" s="72"/>
       <c r="D131" s="10"/>
     </row>
     <row r="132" customHeight="1" spans="1:4">
-      <c r="A132" s="76" t="s">
+      <c r="A132" s="73" t="s">
         <v>210</v>
       </c>
-      <c r="B132" s="77" t="s">
+      <c r="B132" s="74" t="s">
         <v>204</v>
       </c>
-      <c r="C132" s="78">
+      <c r="C132" s="75">
         <v>135</v>
       </c>
       <c r="D132" s="10" t="s">
@@ -4431,11 +4426,11 @@
       </c>
     </row>
     <row r="133" customHeight="1" spans="1:4">
-      <c r="A133" s="74"/>
-      <c r="B133" s="77" t="s">
+      <c r="A133" s="71"/>
+      <c r="B133" s="74" t="s">
         <v>208</v>
       </c>
-      <c r="C133" s="78">
+      <c r="C133" s="75">
         <v>245</v>
       </c>
       <c r="D133" s="10" t="s">
@@ -4443,13 +4438,13 @@
       </c>
     </row>
     <row r="134" ht="46" customHeight="1" spans="1:4">
-      <c r="A134" s="80" t="s">
+      <c r="A134" s="77" t="s">
         <v>213</v>
       </c>
-      <c r="B134" s="81" t="s">
+      <c r="B134" s="78" t="s">
         <v>214</v>
       </c>
-      <c r="C134" s="82">
+      <c r="C134" s="79">
         <v>215</v>
       </c>
       <c r="D134" s="10" t="s">
@@ -4457,51 +4452,51 @@
       </c>
     </row>
     <row r="135" customHeight="1" spans="1:4">
-      <c r="A135" s="83" t="s">
+      <c r="A135" s="80" t="s">
         <v>216</v>
       </c>
-      <c r="B135" s="84" t="s">
+      <c r="B135" s="81" t="s">
         <v>217</v>
       </c>
-      <c r="C135" s="85">
+      <c r="C135" s="82">
         <v>258</v>
       </c>
-      <c r="D135" s="86" t="s">
+      <c r="D135" s="83" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="136" customHeight="1" spans="1:4">
-      <c r="A136" s="83"/>
-      <c r="B136" s="87"/>
-      <c r="C136" s="85"/>
-      <c r="D136" s="88"/>
+      <c r="A136" s="80"/>
+      <c r="B136" s="84"/>
+      <c r="C136" s="82"/>
+      <c r="D136" s="85"/>
     </row>
     <row r="137" customHeight="1" spans="1:4">
-      <c r="A137" s="83"/>
-      <c r="B137" s="87"/>
-      <c r="C137" s="85"/>
-      <c r="D137" s="88"/>
+      <c r="A137" s="80"/>
+      <c r="B137" s="84"/>
+      <c r="C137" s="82"/>
+      <c r="D137" s="85"/>
     </row>
     <row r="138" customHeight="1" spans="1:4">
-      <c r="A138" s="83"/>
-      <c r="B138" s="87"/>
-      <c r="C138" s="85"/>
-      <c r="D138" s="89"/>
+      <c r="A138" s="80"/>
+      <c r="B138" s="84"/>
+      <c r="C138" s="82"/>
+      <c r="D138" s="86"/>
     </row>
     <row r="139" customHeight="1" spans="1:4">
-      <c r="A139" s="90"/>
-      <c r="B139" s="91"/>
-      <c r="C139" s="91"/>
-      <c r="D139" s="92"/>
+      <c r="A139" s="87"/>
+      <c r="B139" s="88"/>
+      <c r="C139" s="88"/>
+      <c r="D139" s="89"/>
     </row>
     <row r="140" customHeight="1" spans="1:4">
-      <c r="A140" s="93" t="s">
+      <c r="A140" s="90" t="s">
         <v>219</v>
       </c>
-      <c r="B140" s="94" t="s">
+      <c r="B140" s="91" t="s">
         <v>220</v>
       </c>
-      <c r="C140" s="95">
+      <c r="C140" s="92">
         <v>10</v>
       </c>
       <c r="D140" s="10" t="s">
@@ -4509,11 +4504,11 @@
       </c>
     </row>
     <row r="141" customHeight="1" spans="1:4">
-      <c r="A141" s="94"/>
-      <c r="B141" s="96" t="s">
+      <c r="A141" s="91"/>
+      <c r="B141" s="93" t="s">
         <v>222</v>
       </c>
-      <c r="C141" s="97">
+      <c r="C141" s="94">
         <v>15</v>
       </c>
       <c r="D141" s="10" t="s">
@@ -4521,13 +4516,13 @@
       </c>
     </row>
     <row r="142" customHeight="1" spans="1:4">
-      <c r="A142" s="93" t="s">
+      <c r="A142" s="90" t="s">
         <v>224</v>
       </c>
-      <c r="B142" s="94" t="s">
+      <c r="B142" s="91" t="s">
         <v>220</v>
       </c>
-      <c r="C142" s="95">
+      <c r="C142" s="92">
         <v>15</v>
       </c>
       <c r="D142" s="10" t="s">
@@ -4535,11 +4530,11 @@
       </c>
     </row>
     <row r="143" customHeight="1" spans="1:4">
-      <c r="A143" s="94"/>
-      <c r="B143" s="96" t="s">
+      <c r="A143" s="91"/>
+      <c r="B143" s="93" t="s">
         <v>222</v>
       </c>
-      <c r="C143" s="97">
+      <c r="C143" s="94">
         <v>20</v>
       </c>
       <c r="D143" s="10" t="s">
@@ -4547,13 +4542,13 @@
       </c>
     </row>
     <row r="144" customHeight="1" spans="1:4">
-      <c r="A144" s="94" t="s">
+      <c r="A144" s="91" t="s">
         <v>227</v>
       </c>
-      <c r="B144" s="96" t="s">
+      <c r="B144" s="93" t="s">
         <v>228</v>
       </c>
-      <c r="C144" s="97">
+      <c r="C144" s="94">
         <v>8</v>
       </c>
       <c r="D144" s="10" t="s">
@@ -4561,408 +4556,408 @@
       </c>
     </row>
     <row r="145" customHeight="1" spans="1:4">
-      <c r="A145" s="96"/>
-      <c r="B145" s="96"/>
-      <c r="C145" s="96"/>
+      <c r="A145" s="93"/>
+      <c r="B145" s="93"/>
+      <c r="C145" s="93"/>
       <c r="D145" s="10"/>
     </row>
     <row r="146" customHeight="1" spans="1:4">
-      <c r="A146" s="96" t="s">
+      <c r="A146" s="93" t="s">
         <v>229</v>
       </c>
-      <c r="B146" s="96"/>
-      <c r="C146" s="96">
+      <c r="B146" s="93"/>
+      <c r="C146" s="93">
         <v>6</v>
       </c>
       <c r="D146" s="10"/>
     </row>
     <row r="147" customHeight="1" spans="1:4">
-      <c r="A147" s="96" t="s">
+      <c r="A147" s="93" t="s">
         <v>230</v>
       </c>
-      <c r="B147" s="96"/>
-      <c r="C147" s="96">
+      <c r="B147" s="93"/>
+      <c r="C147" s="93">
         <v>10</v>
       </c>
       <c r="D147" s="10"/>
     </row>
     <row r="148" customHeight="1" spans="1:4">
-      <c r="A148" s="96" t="s">
+      <c r="A148" s="93" t="s">
         <v>231</v>
       </c>
-      <c r="B148" s="96"/>
-      <c r="C148" s="96">
+      <c r="B148" s="93"/>
+      <c r="C148" s="93">
         <v>40</v>
       </c>
       <c r="D148" s="10"/>
     </row>
     <row r="149" customHeight="1" spans="1:4">
-      <c r="A149" s="96" t="s">
+      <c r="A149" s="93" t="s">
         <v>232</v>
       </c>
-      <c r="B149" s="96"/>
-      <c r="C149" s="96">
+      <c r="B149" s="93"/>
+      <c r="C149" s="93">
         <v>40</v>
       </c>
       <c r="D149" s="10"/>
     </row>
     <row r="150" customHeight="1" spans="1:4">
-      <c r="A150" s="96"/>
-      <c r="B150" s="96"/>
-      <c r="C150" s="96"/>
+      <c r="A150" s="93"/>
+      <c r="B150" s="93"/>
+      <c r="C150" s="93"/>
       <c r="D150" s="10"/>
     </row>
     <row r="151" customHeight="1" spans="1:4">
-      <c r="A151" s="96"/>
-      <c r="B151" s="96"/>
-      <c r="C151" s="96"/>
+      <c r="A151" s="93"/>
+      <c r="B151" s="93"/>
+      <c r="C151" s="93"/>
       <c r="D151" s="10"/>
     </row>
     <row r="152" customHeight="1" spans="1:4">
-      <c r="A152" s="96"/>
-      <c r="B152" s="96"/>
-      <c r="C152" s="96"/>
+      <c r="A152" s="93"/>
+      <c r="B152" s="93"/>
+      <c r="C152" s="93"/>
       <c r="D152" s="10"/>
     </row>
     <row r="153" customHeight="1" spans="1:4">
-      <c r="A153" s="96"/>
-      <c r="B153" s="96"/>
-      <c r="C153" s="96"/>
+      <c r="A153" s="93"/>
+      <c r="B153" s="93"/>
+      <c r="C153" s="93"/>
       <c r="D153" s="10"/>
     </row>
     <row r="154" customHeight="1" spans="1:4">
-      <c r="A154" s="96"/>
-      <c r="B154" s="96"/>
-      <c r="C154" s="96"/>
+      <c r="A154" s="93"/>
+      <c r="B154" s="93"/>
+      <c r="C154" s="93"/>
       <c r="D154" s="10"/>
     </row>
     <row r="155" customHeight="1" spans="1:4">
-      <c r="A155" s="98"/>
-      <c r="B155" s="96"/>
-      <c r="C155" s="96"/>
+      <c r="A155" s="95"/>
+      <c r="B155" s="93"/>
+      <c r="C155" s="93"/>
       <c r="D155" s="10"/>
     </row>
     <row r="156" customHeight="1" spans="1:4">
-      <c r="A156" s="99"/>
-      <c r="B156" s="99"/>
-      <c r="C156" s="100"/>
+      <c r="A156" s="96"/>
+      <c r="B156" s="96"/>
+      <c r="C156" s="97"/>
       <c r="D156" s="10"/>
     </row>
     <row r="157" customHeight="1" spans="1:4">
-      <c r="A157" s="96"/>
-      <c r="B157" s="96"/>
-      <c r="C157" s="97"/>
+      <c r="A157" s="93"/>
+      <c r="B157" s="93"/>
+      <c r="C157" s="94"/>
       <c r="D157" s="10"/>
     </row>
     <row r="158" customHeight="1" spans="1:4">
-      <c r="A158" s="98"/>
-      <c r="B158" s="98"/>
-      <c r="C158" s="101"/>
-      <c r="D158" s="102"/>
+      <c r="A158" s="95"/>
+      <c r="B158" s="95"/>
+      <c r="C158" s="98"/>
+      <c r="D158" s="99"/>
     </row>
     <row r="159" ht="26" customHeight="1" spans="1:4">
-      <c r="A159" s="103"/>
-      <c r="B159" s="103"/>
-      <c r="C159" s="104"/>
-      <c r="D159" s="103"/>
+      <c r="A159" s="100"/>
+      <c r="B159" s="100"/>
+      <c r="C159" s="101"/>
+      <c r="D159" s="100"/>
     </row>
     <row r="160" customHeight="1" spans="1:4">
-      <c r="A160" s="105"/>
-      <c r="B160" s="106"/>
-      <c r="C160" s="107"/>
-      <c r="D160" s="106"/>
+      <c r="A160" s="102"/>
+      <c r="B160" s="103"/>
+      <c r="C160" s="104"/>
+      <c r="D160" s="103"/>
     </row>
     <row r="161" customHeight="1" spans="1:4">
-      <c r="A161" s="108"/>
-      <c r="B161" s="106"/>
-      <c r="C161" s="107"/>
-      <c r="D161" s="106"/>
+      <c r="A161" s="105"/>
+      <c r="B161" s="103"/>
+      <c r="C161" s="104"/>
+      <c r="D161" s="103"/>
     </row>
     <row r="162" customHeight="1" spans="1:4">
-      <c r="A162" s="105"/>
-      <c r="B162" s="106"/>
-      <c r="C162" s="106"/>
-      <c r="D162" s="106"/>
+      <c r="A162" s="102"/>
+      <c r="B162" s="103"/>
+      <c r="C162" s="103"/>
+      <c r="D162" s="103"/>
     </row>
     <row r="163" customHeight="1" spans="1:4">
-      <c r="A163" s="109"/>
-      <c r="B163" s="106"/>
-      <c r="C163" s="106"/>
-      <c r="D163" s="106"/>
+      <c r="A163" s="106"/>
+      <c r="B163" s="103"/>
+      <c r="C163" s="103"/>
+      <c r="D163" s="103"/>
     </row>
     <row r="164" customHeight="1" spans="1:4">
-      <c r="A164" s="109"/>
-      <c r="B164" s="106"/>
-      <c r="C164" s="106"/>
-      <c r="D164" s="106"/>
+      <c r="A164" s="106"/>
+      <c r="B164" s="103"/>
+      <c r="C164" s="103"/>
+      <c r="D164" s="103"/>
     </row>
     <row r="165" customHeight="1" spans="1:4">
-      <c r="A165" s="109"/>
-      <c r="B165" s="106"/>
-      <c r="C165" s="106"/>
-      <c r="D165" s="106"/>
+      <c r="A165" s="106"/>
+      <c r="B165" s="103"/>
+      <c r="C165" s="103"/>
+      <c r="D165" s="103"/>
     </row>
     <row r="166" customHeight="1" spans="1:4">
-      <c r="A166" s="108"/>
-      <c r="B166" s="106"/>
-      <c r="C166" s="106"/>
-      <c r="D166" s="106"/>
+      <c r="A166" s="105"/>
+      <c r="B166" s="103"/>
+      <c r="C166" s="103"/>
+      <c r="D166" s="103"/>
     </row>
     <row r="167" customHeight="1" spans="1:4">
-      <c r="A167" s="109"/>
-      <c r="B167" s="106"/>
-      <c r="C167" s="106"/>
-      <c r="D167" s="106"/>
+      <c r="A167" s="106"/>
+      <c r="B167" s="103"/>
+      <c r="C167" s="103"/>
+      <c r="D167" s="103"/>
     </row>
     <row r="168" customHeight="1" spans="1:4">
-      <c r="A168" s="109"/>
-      <c r="B168" s="106"/>
-      <c r="C168" s="106"/>
-      <c r="D168" s="106"/>
+      <c r="A168" s="106"/>
+      <c r="B168" s="103"/>
+      <c r="C168" s="103"/>
+      <c r="D168" s="103"/>
     </row>
     <row r="169" customHeight="1" spans="1:4">
-      <c r="A169" s="109"/>
-      <c r="B169" s="106"/>
-      <c r="C169" s="106"/>
-      <c r="D169" s="106"/>
+      <c r="A169" s="106"/>
+      <c r="B169" s="103"/>
+      <c r="C169" s="103"/>
+      <c r="D169" s="103"/>
     </row>
     <row r="170" customHeight="1" spans="1:4">
-      <c r="A170" s="108"/>
-      <c r="B170" s="106"/>
-      <c r="C170" s="106"/>
-      <c r="D170" s="106"/>
+      <c r="A170" s="105"/>
+      <c r="B170" s="103"/>
+      <c r="C170" s="103"/>
+      <c r="D170" s="103"/>
     </row>
     <row r="171" customHeight="1" spans="1:4">
-      <c r="A171" s="110"/>
-      <c r="B171" s="111"/>
-      <c r="C171" s="111"/>
-      <c r="D171" s="112"/>
+      <c r="A171" s="107"/>
+      <c r="B171" s="108"/>
+      <c r="C171" s="108"/>
+      <c r="D171" s="109"/>
     </row>
     <row r="172" customHeight="1" spans="1:4">
-      <c r="A172" s="113"/>
-      <c r="B172" s="113"/>
-      <c r="C172" s="114"/>
+      <c r="A172" s="110"/>
+      <c r="B172" s="110"/>
+      <c r="C172" s="111"/>
       <c r="D172" s="10"/>
     </row>
     <row r="173" customHeight="1" spans="1:4">
-      <c r="A173" s="113"/>
-      <c r="B173" s="113"/>
-      <c r="C173" s="114"/>
+      <c r="A173" s="110"/>
+      <c r="B173" s="110"/>
+      <c r="C173" s="111"/>
       <c r="D173" s="10"/>
     </row>
     <row r="174" customHeight="1" spans="1:4">
-      <c r="A174" s="113"/>
-      <c r="B174" s="113"/>
-      <c r="C174" s="114"/>
+      <c r="A174" s="110"/>
+      <c r="B174" s="110"/>
+      <c r="C174" s="111"/>
       <c r="D174" s="10"/>
     </row>
     <row r="175" customHeight="1" spans="1:4">
-      <c r="A175" s="115"/>
-      <c r="B175" s="113"/>
-      <c r="C175" s="116"/>
+      <c r="A175" s="112"/>
+      <c r="B175" s="110"/>
+      <c r="C175" s="113"/>
       <c r="D175" s="10"/>
     </row>
     <row r="176" s="1" customFormat="1" customHeight="1" spans="1:6">
-      <c r="A176" s="117"/>
-      <c r="B176" s="118"/>
-      <c r="C176" s="118"/>
-      <c r="D176" s="119"/>
+      <c r="A176" s="114"/>
+      <c r="B176" s="115"/>
+      <c r="C176" s="115"/>
+      <c r="D176" s="116"/>
       <c r="E176" s="3"/>
-      <c r="F176" s="131"/>
+      <c r="F176" s="128"/>
     </row>
     <row r="177" customHeight="1" spans="1:4">
-      <c r="A177" s="115"/>
-      <c r="B177" s="115"/>
-      <c r="C177" s="116"/>
+      <c r="A177" s="112"/>
+      <c r="B177" s="112"/>
+      <c r="C177" s="113"/>
       <c r="D177" s="10"/>
     </row>
     <row r="178" customHeight="1" spans="1:4">
-      <c r="A178" s="115"/>
-      <c r="B178" s="115"/>
-      <c r="C178" s="116"/>
+      <c r="A178" s="112"/>
+      <c r="B178" s="112"/>
+      <c r="C178" s="113"/>
       <c r="D178" s="10"/>
     </row>
     <row r="179" customHeight="1" spans="1:4">
-      <c r="A179" s="120"/>
-      <c r="B179" s="120"/>
-      <c r="C179" s="116"/>
+      <c r="A179" s="117"/>
+      <c r="B179" s="117"/>
+      <c r="C179" s="113"/>
       <c r="D179" s="10"/>
     </row>
     <row r="180" customHeight="1" spans="1:4">
-      <c r="A180" s="121"/>
-      <c r="B180" s="120"/>
-      <c r="C180" s="120"/>
+      <c r="A180" s="118"/>
+      <c r="B180" s="117"/>
+      <c r="C180" s="117"/>
       <c r="D180" s="10"/>
     </row>
     <row r="181" customHeight="1" spans="1:4">
-      <c r="A181" s="122"/>
-      <c r="B181" s="120"/>
-      <c r="C181" s="120"/>
+      <c r="A181" s="119"/>
+      <c r="B181" s="117"/>
+      <c r="C181" s="117"/>
       <c r="D181" s="10"/>
     </row>
     <row r="182" customHeight="1" spans="1:4">
-      <c r="A182" s="120"/>
-      <c r="B182" s="120"/>
-      <c r="C182" s="120"/>
+      <c r="A182" s="117"/>
+      <c r="B182" s="117"/>
+      <c r="C182" s="117"/>
       <c r="D182" s="10"/>
     </row>
     <row r="183" customHeight="1" spans="1:4">
-      <c r="A183" s="123"/>
-      <c r="B183" s="123"/>
-      <c r="C183" s="123"/>
+      <c r="A183" s="120"/>
+      <c r="B183" s="120"/>
+      <c r="C183" s="120"/>
       <c r="D183" s="10"/>
     </row>
     <row r="184" customHeight="1" spans="1:4">
-      <c r="A184" s="124"/>
-      <c r="B184" s="125"/>
-      <c r="C184" s="125"/>
-      <c r="D184" s="126"/>
+      <c r="A184" s="121"/>
+      <c r="B184" s="122"/>
+      <c r="C184" s="122"/>
+      <c r="D184" s="123"/>
     </row>
     <row r="185" customHeight="1" spans="1:4">
-      <c r="A185" s="127"/>
-      <c r="B185" s="125"/>
-      <c r="C185" s="128"/>
-      <c r="D185" s="126"/>
+      <c r="A185" s="124"/>
+      <c r="B185" s="122"/>
+      <c r="C185" s="125"/>
+      <c r="D185" s="123"/>
     </row>
     <row r="186" customHeight="1" spans="1:4">
-      <c r="A186" s="129"/>
-      <c r="B186" s="125"/>
-      <c r="C186" s="128"/>
-      <c r="D186" s="126"/>
+      <c r="A186" s="126"/>
+      <c r="B186" s="122"/>
+      <c r="C186" s="125"/>
+      <c r="D186" s="123"/>
     </row>
     <row r="187" customHeight="1" spans="1:4">
-      <c r="A187" s="130"/>
-      <c r="B187" s="130"/>
-      <c r="C187" s="130"/>
-      <c r="D187" s="130"/>
+      <c r="A187" s="127"/>
+      <c r="B187" s="127"/>
+      <c r="C187" s="127"/>
+      <c r="D187" s="127"/>
     </row>
     <row r="188" customHeight="1" spans="1:4">
-      <c r="A188" s="130"/>
-      <c r="B188" s="130"/>
-      <c r="C188" s="130"/>
-      <c r="D188" s="130"/>
+      <c r="A188" s="127"/>
+      <c r="B188" s="127"/>
+      <c r="C188" s="127"/>
+      <c r="D188" s="127"/>
     </row>
     <row r="189" customHeight="1" spans="1:4">
-      <c r="A189" s="130"/>
-      <c r="B189" s="130"/>
-      <c r="C189" s="130"/>
-      <c r="D189" s="130"/>
+      <c r="A189" s="127"/>
+      <c r="B189" s="127"/>
+      <c r="C189" s="127"/>
+      <c r="D189" s="127"/>
     </row>
     <row r="190" customHeight="1" spans="1:4">
-      <c r="A190" s="130"/>
-      <c r="B190" s="130"/>
-      <c r="C190" s="130"/>
-      <c r="D190" s="130"/>
+      <c r="A190" s="127"/>
+      <c r="B190" s="127"/>
+      <c r="C190" s="127"/>
+      <c r="D190" s="127"/>
     </row>
     <row r="191" customHeight="1" spans="1:4">
-      <c r="A191" s="130"/>
-      <c r="B191" s="130"/>
-      <c r="C191" s="130"/>
-      <c r="D191" s="130"/>
+      <c r="A191" s="127"/>
+      <c r="B191" s="127"/>
+      <c r="C191" s="127"/>
+      <c r="D191" s="127"/>
     </row>
     <row r="192" customHeight="1" spans="1:4">
-      <c r="A192" s="130"/>
-      <c r="B192" s="130"/>
-      <c r="C192" s="130"/>
-      <c r="D192" s="130"/>
+      <c r="A192" s="127"/>
+      <c r="B192" s="127"/>
+      <c r="C192" s="127"/>
+      <c r="D192" s="127"/>
     </row>
     <row r="193" customHeight="1" spans="1:4">
-      <c r="A193" s="130"/>
-      <c r="B193" s="130"/>
-      <c r="C193" s="130"/>
-      <c r="D193" s="130"/>
+      <c r="A193" s="127"/>
+      <c r="B193" s="127"/>
+      <c r="C193" s="127"/>
+      <c r="D193" s="127"/>
     </row>
     <row r="194" customHeight="1" spans="1:4">
-      <c r="A194" s="130"/>
-      <c r="B194" s="130"/>
-      <c r="C194" s="130"/>
-      <c r="D194" s="130"/>
+      <c r="A194" s="127"/>
+      <c r="B194" s="127"/>
+      <c r="C194" s="127"/>
+      <c r="D194" s="127"/>
     </row>
     <row r="195" ht="97" customHeight="1" spans="1:4">
-      <c r="A195" s="132"/>
-      <c r="B195" s="130"/>
-      <c r="C195" s="130"/>
-      <c r="D195" s="130"/>
+      <c r="A195" s="129"/>
+      <c r="B195" s="127"/>
+      <c r="C195" s="127"/>
+      <c r="D195" s="127"/>
     </row>
     <row r="196" ht="146" customHeight="1" spans="1:4">
-      <c r="A196" s="132"/>
-      <c r="B196" s="130"/>
-      <c r="C196" s="130"/>
-      <c r="D196" s="130"/>
+      <c r="A196" s="129"/>
+      <c r="B196" s="127"/>
+      <c r="C196" s="127"/>
+      <c r="D196" s="127"/>
     </row>
     <row r="197" ht="42" customHeight="1" spans="1:4">
-      <c r="A197" s="130"/>
-      <c r="B197" s="130"/>
-      <c r="C197" s="130"/>
-      <c r="D197" s="130"/>
+      <c r="A197" s="127"/>
+      <c r="B197" s="127"/>
+      <c r="C197" s="127"/>
+      <c r="D197" s="127"/>
     </row>
     <row r="198" ht="133" customHeight="1" spans="1:4">
-      <c r="A198" s="132"/>
-      <c r="B198" s="130"/>
-      <c r="C198" s="130"/>
-      <c r="D198" s="130"/>
+      <c r="A198" s="129"/>
+      <c r="B198" s="127"/>
+      <c r="C198" s="127"/>
+      <c r="D198" s="127"/>
     </row>
     <row r="199" s="2" customFormat="1" ht="149" customHeight="1" spans="1:6">
-      <c r="A199" s="133"/>
-      <c r="B199" s="134"/>
-      <c r="C199" s="134"/>
-      <c r="D199" s="134"/>
-      <c r="E199" s="135"/>
-      <c r="F199" s="135"/>
+      <c r="A199" s="130"/>
+      <c r="B199" s="131"/>
+      <c r="C199" s="131"/>
+      <c r="D199" s="131"/>
+      <c r="E199" s="132"/>
+      <c r="F199" s="132"/>
     </row>
     <row r="200" s="2" customFormat="1" ht="141" customHeight="1" spans="1:6">
-      <c r="A200" s="133"/>
-      <c r="B200" s="134"/>
-      <c r="C200" s="134"/>
-      <c r="D200" s="134"/>
-      <c r="E200" s="135"/>
-      <c r="F200" s="135"/>
+      <c r="A200" s="130"/>
+      <c r="B200" s="131"/>
+      <c r="C200" s="131"/>
+      <c r="D200" s="131"/>
+      <c r="E200" s="132"/>
+      <c r="F200" s="132"/>
     </row>
     <row r="201" ht="106" customHeight="1" spans="1:4">
-      <c r="A201" s="132"/>
-      <c r="B201" s="130"/>
-      <c r="C201" s="130"/>
-      <c r="D201" s="130"/>
+      <c r="A201" s="129"/>
+      <c r="B201" s="127"/>
+      <c r="C201" s="127"/>
+      <c r="D201" s="127"/>
     </row>
     <row r="202" ht="193" customHeight="1" spans="1:4">
-      <c r="A202" s="132"/>
-      <c r="B202" s="130"/>
-      <c r="C202" s="130"/>
-      <c r="D202" s="130"/>
+      <c r="A202" s="129"/>
+      <c r="B202" s="127"/>
+      <c r="C202" s="127"/>
+      <c r="D202" s="127"/>
     </row>
     <row r="203" ht="189" customHeight="1" spans="1:4">
-      <c r="A203" s="132"/>
-      <c r="B203" s="130"/>
-      <c r="C203" s="130"/>
-      <c r="D203" s="130"/>
+      <c r="A203" s="129"/>
+      <c r="B203" s="127"/>
+      <c r="C203" s="127"/>
+      <c r="D203" s="127"/>
     </row>
     <row r="204" ht="136" customHeight="1" spans="1:4">
-      <c r="A204" s="132"/>
-      <c r="B204" s="130"/>
-      <c r="C204" s="130"/>
-      <c r="D204" s="130"/>
+      <c r="A204" s="129"/>
+      <c r="B204" s="127"/>
+      <c r="C204" s="127"/>
+      <c r="D204" s="127"/>
     </row>
     <row r="205" ht="122" customHeight="1" spans="1:4">
-      <c r="A205" s="132"/>
-      <c r="B205" s="130"/>
-      <c r="C205" s="130"/>
-      <c r="D205" s="130"/>
+      <c r="A205" s="129"/>
+      <c r="B205" s="127"/>
+      <c r="C205" s="127"/>
+      <c r="D205" s="127"/>
     </row>
     <row r="206" ht="128" customHeight="1" spans="1:4">
-      <c r="A206" s="132"/>
-      <c r="B206" s="130"/>
-      <c r="C206" s="130"/>
-      <c r="D206" s="130"/>
+      <c r="A206" s="129"/>
+      <c r="B206" s="127"/>
+      <c r="C206" s="127"/>
+      <c r="D206" s="127"/>
     </row>
     <row r="207" ht="164" customHeight="1" spans="1:4">
-      <c r="A207" s="132"/>
-      <c r="B207" s="130"/>
-      <c r="C207" s="130"/>
-      <c r="D207" s="130"/>
+      <c r="A207" s="129"/>
+      <c r="B207" s="127"/>
+      <c r="C207" s="127"/>
+      <c r="D207" s="127"/>
     </row>
     <row r="208" ht="164" customHeight="1"/>
   </sheetData>
-  <mergeCells count="58">
+  <mergeCells count="57">
     <mergeCell ref="A127:D127"/>
     <mergeCell ref="A139:D139"/>
     <mergeCell ref="A171:D171"/>
@@ -4994,7 +4989,6 @@
     <mergeCell ref="A82:A84"/>
     <mergeCell ref="A86:A87"/>
     <mergeCell ref="A89:A92"/>
-    <mergeCell ref="A93:A95"/>
     <mergeCell ref="A96:A97"/>
     <mergeCell ref="A98:A99"/>
     <mergeCell ref="A101:A102"/>

</xml_diff>